<commit_message>
Restore reviewed Jakarta Banten boundary relations
</commit_message>
<xml_diff>
--- a/samples/ss_gucl_ingest.xlsx
+++ b/samples/ss_gucl_ingest.xlsx
@@ -5882,7 +5882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6682,6 +6682,178 @@
       <c r="J21" s="23" t="inlineStr">
         <is>
           <t>Manual audit SLD view kanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SARAN4</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SARAN4 (boundary external)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SRANG</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RGKOT</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>RGKOT (boundary external)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SARAN4</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BUNAR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BUNAR (boundary external)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RGKOT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>KRACAK</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRACAK (boundary spur)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BUNAR</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
         </is>
       </c>
     </row>

</xml_diff>